<commit_message>
Changed the UI and Created the Mentor Login
</commit_message>
<xml_diff>
--- a/users/ck2/Sandhata_Internship_Log.xlsx
+++ b/users/ck2/Sandhata_Internship_Log.xlsx
@@ -785,10 +785,14 @@
           <t>Work</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Done Morning works</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
+      <c r="A9" s="12" t="n"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>11:00</t>
@@ -807,10 +811,14 @@
           <t>Work</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Done Evening things</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
+      <c r="A10" s="12" t="n"/>
       <c r="B10" s="8" t="inlineStr">
         <is>
           <t>13:00</t>
@@ -836,7 +844,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
+      <c r="A11" s="12" t="n"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
           <t>14:00</t>
@@ -858,7 +866,7 @@
       <c r="F11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
+      <c r="A12" s="13" t="n"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
           <t>16:00</t>

</xml_diff>

<commit_message>
Added Student File Module
</commit_message>
<xml_diff>
--- a/users/ck2/Sandhata_Internship_Log.xlsx
+++ b/users/ck2/Sandhata_Internship_Log.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -887,11 +887,130 @@
       </c>
       <c r="F12" s="6" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>19/06/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A13:A17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>